<commit_message>
modifikasi menu payroll & bon
</commit_message>
<xml_diff>
--- a/Master_tarif.xlsx
+++ b/Master_tarif.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Hasil Minggu Ini\Essa-Store-App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{25F2563A-F76A-4D18-92AA-AD406D4C1C8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F797685-57D3-45D2-B1A9-2D1B250A8F88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{CECA2AD4-CD37-44C0-91AC-A97D1185B198}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{CECA2AD4-CD37-44C0-91AC-A97D1185B198}"/>
   </bookViews>
   <sheets>
     <sheet name="SKU_Pengsup" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="796" uniqueCount="796">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="809" uniqueCount="804">
   <si>
     <t>Nomor SKU</t>
   </si>
@@ -2431,6 +2431,30 @@
   </si>
   <si>
     <t>HMD-L</t>
+  </si>
+  <si>
+    <t>Jenis</t>
+  </si>
+  <si>
+    <t>Cost</t>
+  </si>
+  <si>
+    <t>PACK</t>
+  </si>
+  <si>
+    <t>HANGTAG</t>
+  </si>
+  <si>
+    <t>WOVEN</t>
+  </si>
+  <si>
+    <t>HTROPE</t>
+  </si>
+  <si>
+    <t>THREAD</t>
+  </si>
+  <si>
+    <t>AKRILIK</t>
   </si>
 </sst>
 </file>
@@ -2440,7 +2464,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;Rp&quot;#,##0"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2481,6 +2505,13 @@
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -2564,7 +2595,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -2590,6 +2621,8 @@
     <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="40% - Accent3" xfId="2" builtinId="39"/>
@@ -2926,7 +2959,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FD8F914-C444-47BA-9F60-B10F23023A52}">
-  <dimension ref="A1:C770"/>
+  <dimension ref="A1:F770"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.7109375" bestFit="1" customWidth="1"/>
@@ -2935,7 +2968,7 @@
     <col min="4" max="4" width="21.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2945,15 +2978,27 @@
       <c r="C1" s="6" t="s">
         <v>598</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E1" s="11" t="s">
+        <v>796</v>
+      </c>
+      <c r="F1" s="11" t="s">
+        <v>797</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="2"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E2" s="12" t="s">
+        <v>799</v>
+      </c>
+      <c r="F2" s="12">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
@@ -2963,8 +3008,14 @@
       <c r="C3" s="2">
         <v>2000</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E3" s="12" t="s">
+        <v>800</v>
+      </c>
+      <c r="F3" s="12">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>3</v>
       </c>
@@ -2974,8 +3025,14 @@
       <c r="C4" s="2">
         <v>2200</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E4" s="12" t="s">
+        <v>801</v>
+      </c>
+      <c r="F4" s="12">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
@@ -2986,7 +3043,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>5</v>
       </c>
@@ -2997,7 +3054,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>6</v>
       </c>
@@ -3008,7 +3065,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>7</v>
       </c>
@@ -3019,7 +3076,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>8</v>
       </c>
@@ -3030,7 +3087,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>9</v>
       </c>
@@ -3041,7 +3098,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>10</v>
       </c>
@@ -3052,7 +3109,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>11</v>
       </c>
@@ -3063,7 +3120,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>12</v>
       </c>
@@ -3074,7 +3131,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>13</v>
       </c>
@@ -3085,7 +3142,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>14</v>
       </c>
@@ -3096,7 +3153,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>15</v>
       </c>
@@ -9601,97 +9658,139 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96A5A135-A07A-4862-A4A7-EC4AA886D053}">
-  <dimension ref="A1:B659"/>
+  <dimension ref="A1:F659"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" customWidth="1"/>
     <col min="2" max="2" width="31.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>772</v>
       </c>
       <c r="B1" s="10" t="s">
         <v>773</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="E1" s="11" t="s">
+        <v>796</v>
+      </c>
+      <c r="F1" s="11" t="s">
+        <v>797</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>774</v>
       </c>
       <c r="B2" s="8">
         <v>900</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="E2" t="s">
+        <v>798</v>
+      </c>
+      <c r="F2">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>775</v>
       </c>
       <c r="B3" s="8">
         <v>1000</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="E3" t="s">
+        <v>799</v>
+      </c>
+      <c r="F3">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>776</v>
       </c>
       <c r="B4">
         <v>700</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="E4" t="s">
+        <v>800</v>
+      </c>
+      <c r="F4">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>777</v>
       </c>
       <c r="B5">
         <v>1000</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="E5" t="s">
+        <v>801</v>
+      </c>
+      <c r="F5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>778</v>
       </c>
       <c r="B6">
         <v>600</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="E6" t="s">
+        <v>802</v>
+      </c>
+      <c r="F6">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>779</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="E7" t="s">
+        <v>803</v>
+      </c>
+      <c r="F7">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>780</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>781</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>782</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>783</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>784</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>785</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>786</v>
       </c>
@@ -9699,12 +9798,12 @@
         <v>700</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>787</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>788</v>
       </c>

</xml_diff>